<commit_message>
projeciltes among other things
</commit_message>
<xml_diff>
--- a/Assets/Data/DataMichaelWorking.xlsx
+++ b/Assets/Data/DataMichaelWorking.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Structure" sheetId="1" state="visible" r:id="rId3"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="119">
   <si>
     <t xml:space="preserve">Num Code</t>
   </si>
@@ -244,36 +244,8 @@
     <t xml:space="preserve">mage-academy</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">input=</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">population:1|</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">gems:1;
+    <t xml:space="preserve">input=population:1|gems:1;
 output=mage:3</t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">bigger-mage-tower</t>
@@ -329,6 +301,12 @@
     <t xml:space="preserve">Move Speed</t>
   </si>
   <si>
+    <t xml:space="preserve">Attack Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attack Data</t>
+  </si>
+  <si>
     <t xml:space="preserve">knight</t>
   </si>
   <si>
@@ -338,9 +316,19 @@
     <t xml:space="preserve">notes about the unit</t>
   </si>
   <si>
+    <t xml:space="preserve">Melee</t>
+  </si>
+  <si>
     <t xml:space="preserve">archer</t>
   </si>
   <si>
+    <t xml:space="preserve">Ranged</t>
+  </si>
+  <si>
+    <t xml:space="preserve">projectile-speed=3;
+projectile-sprite=arrow</t>
+  </si>
+  <si>
     <t xml:space="preserve">lancer</t>
   </si>
   <si>
@@ -368,10 +356,11 @@
     <t xml:space="preserve">druid</t>
   </si>
   <si>
-    <t xml:space="preserve">debug tool</t>
-  </si>
-  <si>
     <t xml:space="preserve">Nature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">projectile-speed=3;
+projectile-sprite=magic-blast</t>
   </si>
   <si>
     <t xml:space="preserve">dragon-rider</t>
@@ -435,7 +424,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -481,10 +470,17 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="Roboto"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Roboto"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -704,7 +700,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -741,7 +737,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -753,7 +749,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -765,11 +761,43 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -988,7 +1016,7 @@
     <tableColumn id="10" name="Attack Speed"/>
     <tableColumn id="11" name="Attack Range"/>
     <tableColumn id="12" name="Move Speed"/>
-    <tableColumn id="13" name=""/>
+    <tableColumn id="13" name="Attack Type"/>
   </tableColumns>
 </table>
 </file>
@@ -1179,7 +1207,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="24.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="1" width="14.43"/>
@@ -1223,7 +1251,7 @@
       <c r="M1" s="3"/>
       <c r="N1" s="5"/>
     </row>
-    <row r="2" customFormat="false" ht="27.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="n">
         <v>1</v>
       </c>
@@ -2228,11 +2256,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr defaultColWidth="8.75390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.57"/>
@@ -2241,10 +2269,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="16.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="14.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="14.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="25.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="38.47"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2281,23 +2310,28 @@
       <c r="L1" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="M1" s="2"/>
+      <c r="M1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D2" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E2" s="7" t="s">
         <v>83</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>81</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>12</v>
@@ -2320,23 +2354,26 @@
       <c r="L2" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="M2" s="6"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M2" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="N2" s="15"/>
+    </row>
+    <row r="3" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>82</v>
-      </c>
       <c r="D3" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>12</v>
@@ -2359,23 +2396,28 @@
       <c r="L3" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="M3" s="13"/>
+      <c r="M3" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="N3" s="16" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>83</v>
-      </c>
       <c r="E4" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>12</v>
@@ -2398,23 +2440,26 @@
       <c r="L4" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="M4" s="6"/>
+      <c r="M4" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="N4" s="15"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>12</v>
@@ -2437,23 +2482,26 @@
       <c r="L5" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="M5" s="13"/>
+      <c r="M5" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="N5" s="16"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>12</v>
@@ -2476,23 +2524,26 @@
       <c r="L6" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="M6" s="6"/>
+      <c r="M6" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="N6" s="15"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>12</v>
@@ -2515,23 +2566,26 @@
       <c r="L7" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="M7" s="13"/>
+      <c r="M7" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="N7" s="16"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>12</v>
@@ -2554,23 +2608,26 @@
       <c r="L8" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="M8" s="6"/>
+      <c r="M8" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="N8" s="15"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F9" s="7" t="s">
         <v>38</v>
@@ -2593,23 +2650,26 @@
       <c r="L9" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="M9" s="13"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M9" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="N9" s="16"/>
+    </row>
+    <row r="10" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>12</v>
@@ -2632,23 +2692,28 @@
       <c r="L10" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="M10" s="6"/>
+      <c r="M10" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="N10" s="19" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>32</v>
@@ -2671,26 +2736,29 @@
       <c r="L11" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="M11" s="13"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M11" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="N11" s="20"/>
+    </row>
+    <row r="12" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="G12" s="7" t="n">
         <v>1</v>
@@ -2710,23 +2778,28 @@
       <c r="L12" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="M12" s="6"/>
+      <c r="M12" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="N12" s="19" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>38</v>
@@ -2749,23 +2822,26 @@
       <c r="L13" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="M13" s="13"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M13" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="N13" s="16"/>
+    </row>
+    <row r="14" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="F14" s="7" t="s">
         <v>35</v>
@@ -2788,23 +2864,28 @@
       <c r="L14" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="M14" s="6"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M14" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="N14" s="19" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>32</v>
@@ -2827,23 +2908,28 @@
       <c r="L15" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="M15" s="13"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M15" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="N15" s="22" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="n">
         <v>15</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>35</v>
@@ -2866,7 +2952,15 @@
       <c r="L16" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="M16" s="6"/>
+      <c r="M16" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="N16" s="19" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N17" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2895,35 +2989,35 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="15" t="s">
+      <c r="A1" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="23" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -2952,7 +3046,7 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="23" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2994,296 +3088,296 @@
   <sheetFormatPr defaultColWidth="12.8046875" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
-        <v>103</v>
-      </c>
-      <c r="B1" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="C1" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="E1" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="F1" s="16" t="s">
+      <c r="A1" s="24" t="s">
         <v>108</v>
       </c>
+      <c r="B1" s="24" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="D1" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="E1" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="F1" s="24" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>92</v>
+      <c r="A2" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>97</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="19"/>
+      <c r="E2" s="27"/>
       <c r="F2" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="20" t="s">
-        <v>81</v>
+      <c r="A3" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="28" t="s">
+        <v>83</v>
       </c>
       <c r="D3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="21"/>
+      <c r="E3" s="29"/>
       <c r="F3" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17" t="n">
+      <c r="A4" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>81</v>
+      <c r="B4" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="28" t="s">
+        <v>83</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="21" t="s">
-        <v>84</v>
+      <c r="E4" s="29" t="s">
+        <v>87</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="n">
+      <c r="A5" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B5" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="20" t="s">
-        <v>81</v>
+      <c r="C5" s="28" t="s">
+        <v>83</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="21" t="s">
-        <v>84</v>
+      <c r="E5" s="29" t="s">
+        <v>87</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="n">
+      <c r="A6" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="20" t="s">
-        <v>81</v>
+      <c r="C6" s="28" t="s">
+        <v>83</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="21" t="s">
-        <v>84</v>
+      <c r="E6" s="29" t="s">
+        <v>87</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="n">
+      <c r="A7" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="20" t="s">
-        <v>81</v>
+      <c r="C7" s="28" t="s">
+        <v>83</v>
       </c>
       <c r="D7" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="21" t="s">
-        <v>84</v>
+      <c r="E7" s="29" t="s">
+        <v>87</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="n">
+      <c r="A8" s="25" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="17" t="n">
+      <c r="B8" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="C8" s="20" t="s">
-        <v>81</v>
+      <c r="C8" s="28" t="s">
+        <v>83</v>
       </c>
       <c r="D8" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="E8" s="21" t="s">
-        <v>84</v>
+      <c r="E8" s="29" t="s">
+        <v>87</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="n">
+      <c r="A9" s="25" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="17" t="n">
+      <c r="B9" s="25" t="n">
         <v>7</v>
       </c>
-      <c r="C9" s="20" t="s">
-        <v>81</v>
+      <c r="C9" s="28" t="s">
+        <v>83</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="E9" s="21" t="s">
-        <v>84</v>
+      <c r="E9" s="29" t="s">
+        <v>87</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="n">
+      <c r="A10" s="25" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="17" t="n">
+      <c r="B10" s="25" t="n">
         <v>8</v>
       </c>
-      <c r="C10" s="20" t="s">
-        <v>81</v>
+      <c r="C10" s="28" t="s">
+        <v>83</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="E10" s="21" t="s">
-        <v>84</v>
+      <c r="E10" s="29" t="s">
+        <v>87</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="17" t="n">
+      <c r="A11" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="25" t="n">
         <v>9</v>
       </c>
-      <c r="C11" s="20" t="s">
-        <v>81</v>
+      <c r="C11" s="28" t="s">
+        <v>83</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="E11" s="21" t="s">
-        <v>84</v>
+      <c r="E11" s="29" t="s">
+        <v>87</v>
       </c>
       <c r="F11" s="1" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="n">
+      <c r="A12" s="25" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="17" t="n">
-        <v>10</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>81</v>
+      <c r="B12" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" s="28" t="s">
+        <v>83</v>
       </c>
       <c r="D12" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="E12" s="21" t="s">
-        <v>84</v>
+      <c r="E12" s="29" t="s">
+        <v>87</v>
       </c>
       <c r="F12" s="1" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17" t="n">
+      <c r="A13" s="25" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="17" t="n">
+      <c r="B13" s="25" t="n">
         <v>11</v>
       </c>
-      <c r="C13" s="20" t="s">
-        <v>81</v>
+      <c r="C13" s="28" t="s">
+        <v>83</v>
       </c>
       <c r="D13" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="E13" s="21" t="s">
-        <v>84</v>
+      <c r="E13" s="29" t="s">
+        <v>87</v>
       </c>
       <c r="F13" s="1" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="n">
+      <c r="A14" s="25" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="17" t="n">
+      <c r="B14" s="25" t="n">
         <v>12</v>
       </c>
-      <c r="C14" s="20" t="s">
-        <v>81</v>
+      <c r="C14" s="28" t="s">
+        <v>83</v>
       </c>
       <c r="D14" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="E14" s="21" t="s">
-        <v>84</v>
+      <c r="E14" s="29" t="s">
+        <v>87</v>
       </c>
       <c r="F14" s="1" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17" t="n">
+      <c r="A15" s="25" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="17" t="n">
+      <c r="B15" s="25" t="n">
         <v>13</v>
       </c>
-      <c r="C15" s="20" t="s">
-        <v>81</v>
+      <c r="C15" s="28" t="s">
+        <v>83</v>
       </c>
       <c r="D15" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="E15" s="21" t="s">
-        <v>84</v>
+      <c r="E15" s="29" t="s">
+        <v>87</v>
       </c>
       <c r="F15" s="1" t="n">
         <v>8</v>
@@ -3317,23 +3411,23 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="B1" s="16" t="s">
+      <c r="A1" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="C1" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="E1" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="F1" s="16" t="s">
-        <v>113</v>
+      <c r="B1" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1" s="24" t="s">
+        <v>115</v>
+      </c>
+      <c r="D1" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="E1" s="24" t="s">
+        <v>117</v>
+      </c>
+      <c r="F1" s="24" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3483,7 +3577,7 @@
       <c r="B9" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C9" s="30" t="n">
         <v>0.6</v>
       </c>
       <c r="D9" s="1" t="n">
@@ -3523,7 +3617,7 @@
       <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="30" t="n">
         <v>0.6</v>
       </c>
       <c r="D11" s="1" t="n">
@@ -3563,7 +3657,7 @@
       <c r="B13" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C13" s="22" t="n">
+      <c r="C13" s="30" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="1" t="n">
@@ -3603,7 +3697,7 @@
       <c r="B15" s="1" t="n">
         <v>0.6</v>
       </c>
-      <c r="C15" s="22" t="n">
+      <c r="C15" s="30" t="n">
         <v>1</v>
       </c>
       <c r="D15" s="1" t="n">
@@ -3620,7 +3714,7 @@
       <c r="A16" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="22" t="n">
+      <c r="B16" s="30" t="n">
         <v>0.6</v>
       </c>
       <c r="C16" s="1" t="n">
@@ -3643,7 +3737,7 @@
       <c r="B17" s="1" t="n">
         <v>0.6</v>
       </c>
-      <c r="C17" s="22" t="n">
+      <c r="C17" s="30" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="1" t="n">
@@ -3660,7 +3754,7 @@
       <c r="A18" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="22" t="n">
+      <c r="B18" s="30" t="n">
         <v>0.6</v>
       </c>
       <c r="C18" s="1" t="n">
@@ -3683,7 +3777,7 @@
       <c r="B19" s="1" t="n">
         <v>0.6</v>
       </c>
-      <c r="C19" s="22" t="n">
+      <c r="C19" s="30" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="n">
@@ -3700,7 +3794,7 @@
       <c r="A20" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="22" t="n">
+      <c r="B20" s="30" t="n">
         <v>0.6</v>
       </c>
       <c r="C20" s="1" t="n">

</xml_diff>